<commit_message>
chore: sync templates with esqlabsR and extend config handling
Co-authored-by: KatrinCoboeken <28564329+KatrinCoboeken@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/inst/templates/Individuals.xlsx
+++ b/inst/templates/Individuals.xlsx
@@ -1,121 +1,126 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub repositories\ESQlabs\esqlabsR\inst\extdata\examples\TestProject\Configurations\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD5A8B5-3806-48FE-A083-EFB6E2032A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="IndividualBiometrics" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="template_Ind" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="IndividualBiometrics" sheetId="1" r:id="rId1"/>
+    <sheet name="Indiv1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
-  <si>
-    <t xml:space="preserve">IndividualId</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Species</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Population</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gender</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight [kg]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Height [cm]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age [year(s)]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protein Ontogenies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MALE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Human</t>
-  </si>
-  <si>
-    <t xml:space="preserve">European_ICRP_2002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FEMALE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Container Path</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organism|Kidney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GFR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ml/min</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>Human</t>
+  </si>
+  <si>
+    <t>European_ICRP_2002</t>
+  </si>
+  <si>
+    <t>IndividualId</t>
+  </si>
+  <si>
+    <t>Species</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Population</t>
+  </si>
+  <si>
+    <t>Weight [kg]</t>
+  </si>
+  <si>
+    <t>Height [cm]</t>
+  </si>
+  <si>
+    <t>Age [year(s)]</t>
+  </si>
+  <si>
+    <t>MALE</t>
+  </si>
+  <si>
+    <t>Indiv1</t>
+  </si>
+  <si>
+    <t>ml/min</t>
+  </si>
+  <si>
+    <t>GFR</t>
+  </si>
+  <si>
+    <t>Organism|Kidney</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Parameter Name</t>
+  </si>
+  <si>
+    <t>Container Path</t>
+  </si>
+  <si>
+    <t>Protein Ontogenies</t>
+  </si>
+  <si>
+    <t>CYP3A4:CYP3A4,CYP2D6:CYP2C8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -127,7 +132,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -135,149 +140,187 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal 2" xfId="20"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{FC690C68-0E55-48A3-908A-41ADC76A33D8}"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -285,24 +328,33 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -315,7 +367,13 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -325,13 +383,15 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
+            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
+                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -339,6 +399,7 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
+                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -346,176 +407,156 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2">
         <v>73</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2">
         <v>176</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="0" t="n">
-        <v>65</v>
-      </c>
-      <c r="F3" s="0" t="n">
-        <v>165</v>
-      </c>
-      <c r="G3" s="0" t="n">
-        <v>30</v>
+      <c r="H2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3892D2-FAF9-44EE-B239-FAC53541F5B5}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.57"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="2" style="1" width="8.71"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="1">
         <v>90</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010011DB5BA7A27696418C6D2C8B46A68E83" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="151fa1d8706c0355297f81811bd06e6b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="398d2b5b-77f8-4c5f-a794-3d35ce849315" xmlns:ns3="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="85a3e53823607994162d1630ec2e7479" ns2:_="" ns3:_="">
     <xsd:import namespace="398d2b5b-77f8-4c5f-a794-3d35ce849315"/>
@@ -752,15 +793,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -773,6 +805,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78CA0B51-7456-4883-901E-100C95177B36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1713C675-E25A-461C-9068-CC8E8BA72888}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -791,14 +831,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78CA0B51-7456-4883-901E-100C95177B36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{028903B1-0B22-4BE6-8A73-043144867A27}">
   <ds:schemaRefs>

</xml_diff>